<commit_message>
Update binary files and delete outdated DPR Excel files
- Updated multiple binary files including `ErectionCompiled_Output.xlsx`, `ProdDailyExpandedSingles.parquet`, `ProjectDetails.parquet`, `RawData.parquet`, `StringingCompiled_Output.xlsx`, and `StringingCompiled.parquet` to reflect recent changes in data processing.
- Deleted several outdated DPR Excel files to streamline the project directory.
</commit_message>
<xml_diff>
--- a/Raw Data/Projects_KV.xlsx
+++ b/Raw Data/Projects_KV.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9054DEAF-3EA8-4F11-AF1C-3B5D722B8F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27B5637E-0DC8-4148-9864-A7B9BF085760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -114,12 +114,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -149,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -157,6 +163,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,10 +444,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -450,71 +457,95 @@
       <c r="D1" s="2"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
         <v>765</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2" s="3">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3">
         <v>765</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F3" s="3">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>15</v>
       </c>
       <c r="B4">
         <v>765</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F4" s="3">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
         <v>765</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F5" s="3">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6">
         <v>765</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F6">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>2</v>
       </c>
       <c r="B7">
         <v>765</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F7" s="3">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8">
         <v>765</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F8">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9">
         <v>400</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F9" s="3">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -522,7 +553,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -530,7 +561,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -538,7 +569,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -546,7 +577,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -554,7 +585,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>3</v>
       </c>
@@ -562,7 +593,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>

</xml_diff>